<commit_message>
Atualização automática via Dashboard/PAD
</commit_message>
<xml_diff>
--- a/energia.xlsx
+++ b/energia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alyss\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F3F6D8D-594D-4E58-B67B-6AE79F5FA7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2845" documentId="13_ncr:1_{5F541AEE-34E0-4010-BD7A-1C5EA974EAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{483742A9-EB2F-4AD4-9686-88BCB8ED6BBC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55158,6 +55158,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="6a022168024afc72da6ea3dc509b0a8f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a9a89a50b7dc5582b87a24cd504aca59" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -55392,28 +55412,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD397AEE-6A9A-4FE5-A80F-F3820F88B792}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62D13B68-A133-49F3-B106-97FAB6641D90}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -55421,5 +55421,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62D13B68-A133-49F3-B106-97FAB6641D90}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD397AEE-6A9A-4FE5-A80F-F3820F88B792}"/>
 </file>
</xml_diff>